<commit_message>
updated mdl, cdrdfrcp, csc, bs, vsbs
</commit_message>
<xml_diff>
--- a/InputData/elec/CDRDfRCP/Cln Dsptchble Rsrc Dmnd for Rlbty Curve Param.xlsx
+++ b/InputData/elec/CDRDfRCP/Cln Dsptchble Rsrc Dmnd for Rlbty Curve Param.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robbie\Dropbox (Energy Innovation)\My Documents\Energy Policy Solutions\US\Models\eps-us\InputData\elec\CDRDfRCP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\RMI\RMI_all_states\CT\elec\CDRDfRCP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0C0A9FB-66F9-47E6-BEC9-2D0B0D7D12BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{807BDD75-E329-4A58-A125-B99DA39A6A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8520" yWindow="2740" windowWidth="28800" windowHeight="15540" activeTab="1" xr2:uid="{DDCF7A3C-4581-48BB-A680-D5CBB461C8EB}"/>
+    <workbookView xWindow="18375" yWindow="705" windowWidth="8475" windowHeight="16185" xr2:uid="{DDCF7A3C-4581-48BB-A680-D5CBB461C8EB}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>CDRDfRCP Clean Dispatchable Resource Demand for Reliabilty Curve Paramaters</t>
   </si>
@@ -64,6 +64,9 @@
   </si>
   <si>
     <t>required share peak</t>
+  </si>
+  <si>
+    <t>Connecticut</t>
   </si>
 </sst>
 </file>
@@ -107,9 +110,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -424,15 +428,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B207133-CFE8-4DB4-95CD-9BA248AF1C6C}">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="2">
+        <v>45267</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -440,12 +450,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -453,7 +463,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>6</v>
       </c>
@@ -469,28 +479,28 @@
     <tabColor theme="3" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>7</v>
       </c>
       <c r="B1">
-        <v>-11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
       <c r="B2">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>

</xml_diff>